<commit_message>
Fix blog checklist wording
</commit_message>
<xml_diff>
--- a/assets/downloads/2026-03-16-unexpected-exception-exit-or-continue-checklist.xlsx
+++ b/assets/downloads/2026-03-16-unexpected-exception-exit-or-continue-checklist.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Checklist-en" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist-ja'!$A$1:$E$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Checklist-en'!$A$1:$E$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist-ja'!$A$1:$E$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Checklist-en'!$A$1:$E$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,12 +446,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="96" customWidth="1" min="3" max="3"/>
+    <col width="98" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
   </cols>
@@ -491,12 +491,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>継続してよい条件</t>
+          <t>????</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>失敗単位が明確: 1 操作、1 画面、1 ジョブ、1 接続など、捨てる単位が分かる</t>
+          <t>????? 1 ?? / 1 ?? / 1 ??? / 1 ??????????????</t>
         </is>
       </c>
       <c r="D2" s="2" t="n"/>
@@ -510,12 +510,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>継続してよい条件</t>
+          <t>????</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>状態を捨てられる: 破棄して作り直せる、または未反映として扱える</t>
+          <t>??????????????????</t>
         </is>
       </c>
       <c r="D3" s="2" t="n"/>
@@ -529,12 +529,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>継続してよい条件</t>
+          <t>????</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>共有状態が守られる: 他の機能へ汚染が広がらない</t>
+          <t>??????????????????????</t>
         </is>
       </c>
       <c r="D4" s="2" t="n"/>
@@ -548,12 +548,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>継続してよい条件</t>
+          <t>????</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>外部副作用を説明できる: 送った / 送っていない / 再送してよい、が分かる</t>
+          <t>???????????????????</t>
         </is>
       </c>
       <c r="D5" s="2" t="n"/>
@@ -567,12 +567,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>継続してよい条件</t>
+          <t>????</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>利用者へ正直に伝えられる: 「今回の処理は失敗した」と表示できる</t>
+          <t>?????????????????????????</t>
         </is>
       </c>
       <c r="D6" s="2" t="n"/>
@@ -586,12 +586,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>継続してよい条件</t>
+          <t>????</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>監視できる: ログ、メトリクス、ダンプで後追い調査できる</t>
+          <t>?? / ????? / ??????????????</t>
         </is>
       </c>
       <c r="D7" s="2" t="n"/>
@@ -605,12 +605,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>終了したほうがよい条件</t>
+          <t>????</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>途中まで何を変更したか分からない</t>
+          <t>??????????????????????????</t>
         </is>
       </c>
       <c r="D8" s="2" t="n"/>
@@ -624,12 +624,12 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>終了したほうがよい条件</t>
+          <t>????</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>共有の書き換え可能な状態を触っていて、整合が読めない</t>
+          <t>????????????????????????????????</t>
         </is>
       </c>
       <c r="D9" s="2" t="n"/>
@@ -643,12 +643,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>終了したほうがよい条件</t>
+          <t>????</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>ロック、キュー、スレッド、監視ループの寿命管理が壊れた</t>
+          <t>??? / ??? / ???? / ??????????????????????????</t>
         </is>
       </c>
       <c r="D10" s="2" t="n"/>
@@ -662,12 +662,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>終了したほうがよい条件</t>
+          <t>????</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>外部副作用の重複 / 欠落 / 半端が説明できない</t>
+          <t>???????? / ?? / ?????????????????????</t>
         </is>
       </c>
       <c r="D11" s="2" t="n"/>
@@ -681,12 +681,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>終了したほうがよい条件</t>
+          <t>????</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>起動処理や中核インフラの初期化で失敗した</t>
+          <t>????????????????????????????????</t>
         </is>
       </c>
       <c r="D12" s="2" t="n"/>
@@ -700,12 +700,12 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>終了したほうがよい条件</t>
+          <t>????</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>ネイティブ境界やメモリ破壊を疑う</t>
+          <t>?????????????????????????????</t>
         </is>
       </c>
       <c r="D13" s="2" t="n"/>
@@ -719,12 +719,12 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>よくあるNG</t>
+          <t>????</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>catch (Exception) でログだけ出して続ける</t>
+          <t>catch (Exception) ???????????????</t>
         </is>
       </c>
       <c r="D14" s="2" t="n"/>
@@ -738,12 +738,12 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>よくあるNG</t>
+          <t>????</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>最後の未処理例外ハンドラで回復しようとする</t>
+          <t>????????????????????????????</t>
         </is>
       </c>
       <c r="D15" s="2" t="n"/>
@@ -757,12 +757,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>よくあるNG</t>
+          <t>????</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>外部副作用があるのに安易に retry する</t>
+          <t>???????????????????? retry ?????</t>
         </is>
       </c>
       <c r="D16" s="2" t="n"/>
@@ -776,12 +776,12 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>よくあるNG</t>
+          <t>????</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>監視ループが死んだのに UI だけ残す</t>
+          <t>???????????? UI ?????????????</t>
         </is>
       </c>
       <c r="D17" s="2" t="n"/>
@@ -795,12 +795,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>よくあるNG</t>
+          <t>????</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>落とす設計をしていないのに「落としたくない」と言う</t>
+          <t>??????????????? / ??????? / ???? / ?????? / ??????????????</t>
         </is>
       </c>
       <c r="D18" s="2" t="n"/>
@@ -814,12 +814,12 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>判断の順番</t>
+          <t>????</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>失敗した単位を捨てられるか</t>
+          <t>catch ????? UI ???? / 1 ????? / 1 ??? / 1 ?? / ????????????</t>
         </is>
       </c>
       <c r="D19" s="2" t="n"/>
@@ -833,12 +833,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>判断の順番</t>
+          <t>????</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>共有状態を戻せるか、作り直せるか</t>
+          <t>????????????????????</t>
         </is>
       </c>
       <c r="D20" s="2" t="n"/>
@@ -852,12 +852,12 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>判断の順番</t>
+          <t>????</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>外部副作用を説明できるか</t>
+          <t>?????????????????????</t>
         </is>
       </c>
       <c r="D21" s="2" t="n"/>
@@ -871,19 +871,133 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>判断の順番</t>
+          <t>????</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>メモリ / スレッド / ネイティブ境界の健全性は信用できるか</t>
+          <t>??????????????????</t>
         </is>
       </c>
       <c r="D22" s="2" t="n"/>
       <c r="E22" s="2" t="n"/>
     </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>????</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>???????????????????????</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>????</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>WPF / WinForms ????????????????? = ???????????</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>???</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>???????????????????????</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>???</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>???????????????????????</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>???</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>???????????????????</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>???</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>??? / ???? / ?????????????????????</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E22"/>
+  <autoFilter ref="A1:E28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -894,12 +1008,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="96" customWidth="1" min="3" max="3"/>
+    <col width="98" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
   </cols>
@@ -939,12 +1053,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Conditions that support continuation</t>
+          <t>Continuation readiness</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>the failed unit is explicit: one operation, one screen, one job, one connection</t>
+          <t>The failed unit is contained to one operation, one screen, one job, one connection, or a similarly clear boundary</t>
         </is>
       </c>
       <c r="D2" s="2" t="n"/>
@@ -958,12 +1072,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Conditions that support continuation</t>
+          <t>Continuation readiness</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>the damaged state can be thrown away: discard and recreate, or treat as not committed</t>
+          <t>The affected state can be discarded and rebuilt after the exception</t>
         </is>
       </c>
       <c r="D3" s="2" t="n"/>
@@ -977,12 +1091,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Conditions that support continuation</t>
+          <t>Continuation readiness</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>shared state remains protected: the damage does not spread through the rest of the app</t>
+          <t>Damage does not spread into shared mutable state</t>
         </is>
       </c>
       <c r="D4" s="2" t="n"/>
@@ -996,12 +1110,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Conditions that support continuation</t>
+          <t>Continuation readiness</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>external side effects are understandable: you know whether something was sent, committed, or needs retry</t>
+          <t>External side effects and retry safety can still be explained</t>
         </is>
       </c>
       <c r="D5" s="2" t="n"/>
@@ -1015,12 +1129,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Conditions that support continuation</t>
+          <t>Continuation readiness</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>the user can be told the truth: "this operation failed" is a valid message</t>
+          <t>The user can be told honestly that this operation failed</t>
         </is>
       </c>
       <c r="D6" s="2" t="n"/>
@@ -1034,12 +1148,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Conditions that support continuation</t>
+          <t>Continuation readiness</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>the failure can be observed later: logs, metrics, dumps, or other diagnostics exist</t>
+          <t>Logs, metrics, dumps, or similar diagnostics exist for follow-up investigation</t>
         </is>
       </c>
       <c r="D7" s="2" t="n"/>
@@ -1053,12 +1167,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Conditions that support exit</t>
+          <t>Exit readiness</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>you do not know what changed partway</t>
+          <t>The app does not continue when it is unclear what changed partway through</t>
         </is>
       </c>
       <c r="D8" s="2" t="n"/>
@@ -1072,12 +1186,12 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Conditions that support exit</t>
+          <t>Exit readiness</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>shared mutable state may already be inconsistent</t>
+          <t>The app leans toward exit when shared mutable state may already be inconsistent</t>
         </is>
       </c>
       <c r="D9" s="2" t="n"/>
@@ -1091,12 +1205,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Conditions that support exit</t>
+          <t>Exit readiness</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>locks, queues, threads, or loop lifetimes may be broken</t>
+          <t>The app leans toward exit when locks, queues, threads, or monitoring-loop lifetimes may be broken</t>
         </is>
       </c>
       <c r="D10" s="2" t="n"/>
@@ -1110,12 +1224,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Conditions that support exit</t>
+          <t>Exit readiness</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>external side effects are partial or ambiguous</t>
+          <t>The app leans toward exit when duplicated, missing, or partial external side effects cannot be explained</t>
         </is>
       </c>
       <c r="D11" s="2" t="n"/>
@@ -1129,12 +1243,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Conditions that support exit</t>
+          <t>Exit readiness</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>startup or core infrastructure failed</t>
+          <t>Startup or core-infrastructure initialization failures are not hidden behind a partial startup</t>
         </is>
       </c>
       <c r="D12" s="2" t="n"/>
@@ -1148,12 +1262,12 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Conditions that support exit</t>
+          <t>Exit readiness</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>the exception suggests memory or native-boundary corruption</t>
+          <t>Suspected native-boundary damage or memory corruption is not treated as a continue-by-default case</t>
         </is>
       </c>
       <c r="D13" s="2" t="n"/>
@@ -1167,12 +1281,12 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Common bad patterns</t>
+          <t>Implementation policy</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Catch everything, log it, and continue</t>
+          <t>The app does not simply catch Exception, log it, and continue</t>
         </is>
       </c>
       <c r="D14" s="2" t="n"/>
@@ -1186,12 +1300,12 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Common bad patterns</t>
+          <t>Implementation policy</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Treat the final unhandled-exception hook as a recovery point</t>
+          <t>The final unhandled-exception hook is not treated as a recovery point</t>
         </is>
       </c>
       <c r="D15" s="2" t="n"/>
@@ -1205,12 +1319,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Common bad patterns</t>
+          <t>Implementation policy</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Retry blindly when external side effects already happened</t>
+          <t>Operations with external side effects are not retried blindly without replay safety</t>
         </is>
       </c>
       <c r="D16" s="2" t="n"/>
@@ -1224,12 +1338,12 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Common bad patterns</t>
+          <t>Implementation policy</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Leave the UI alive after the real worker died</t>
+          <t>The UI is not kept alive after a real monitoring or worker loop has already died</t>
         </is>
       </c>
       <c r="D17" s="2" t="n"/>
@@ -1243,12 +1357,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Common bad patterns</t>
+          <t>Implementation policy</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Say "we must not crash" without designing for crash</t>
+          <t>If avoiding crashes is important, restart, session recovery, saved progress, replay safety, and failure-domain separation are designed first</t>
         </is>
       </c>
       <c r="D18" s="2" t="n"/>
@@ -1262,12 +1376,12 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Decision order</t>
+          <t>Implementation policy</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Can the failed unit be discarded?</t>
+          <t>Catch points are placed at UI, request, job, connection, or process boundaries rather than everywhere</t>
         </is>
       </c>
       <c r="D19" s="2" t="n"/>
@@ -1281,12 +1395,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Decision order</t>
+          <t>Implementation policy</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Can shared state be repaired or rebuilt?</t>
+          <t>Expected failures and unexpected failures are handled as different categories</t>
         </is>
       </c>
       <c r="D20" s="2" t="n"/>
@@ -1300,12 +1414,12 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Decision order</t>
+          <t>Implementation policy</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Can the external side effects still be explained?</t>
+          <t>Shared mutable state is kept as small as practical</t>
         </is>
       </c>
       <c r="D21" s="2" t="n"/>
@@ -1319,19 +1433,133 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Decision order</t>
+          <t>Implementation policy</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Can memory, threads, and native boundaries still be trusted?</t>
+          <t>Risky work is isolated into another process when the blast radius should stay small</t>
         </is>
       </c>
       <c r="D22" s="2" t="n"/>
       <c r="E22" s="2" t="n"/>
     </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Implementation policy</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Unhandled-exception hooks prioritize recording and diagnostics over fake recovery</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Implementation policy</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>WPF or WinForms unhandled-exception events are not treated as proof that continued execution is safe</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Decision order</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>The first check is whether the failed unit can be discarded</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Decision order</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>The next check is whether shared state can be repaired or rebuilt</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Decision order</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>The next check is whether external side effects can still be explained</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Decision order</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>The last check is whether memory, threads, and native boundaries are still trustworthy</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E22"/>
+  <autoFilter ref="A1:E28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix checklist Excel mojibake
</commit_message>
<xml_diff>
--- a/assets/downloads/2026-03-16-unexpected-exception-exit-or-continue-checklist.xlsx
+++ b/assets/downloads/2026-03-16-unexpected-exception-exit-or-continue-checklist.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -491,12 +491,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>継続判断</t>
+          <t>継続条件</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>失敗した単位が 1 操作 / 1 画面 / 1 ジョブ / 1 接続などの明確な境界に閉じ込められている</t>
+          <t>失敗単位が 1 操作 / 1 画面 / 1 ジョブ / 1 接続などの明確な境界に閉じている</t>
         </is>
       </c>
       <c r="D2" s="2" t="n"/>
@@ -510,12 +510,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>継続判断</t>
+          <t>継続条件</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>例外後に、影響を受けた状態を破棄して作り直せる</t>
+          <t>例外後に、影響を受けた状態を破棄して再構築できる</t>
         </is>
       </c>
       <c r="D3" s="2" t="n"/>
@@ -529,12 +529,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>継続判断</t>
+          <t>継続条件</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>共有の書き換え可能な状態へ汚染が広がらない</t>
+          <t>破損が共有の可変状態へ広がっていない</t>
         </is>
       </c>
       <c r="D4" s="2" t="n"/>
@@ -548,12 +548,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>継続判断</t>
+          <t>継続条件</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>外部副作用の状況と retry の安全性を説明できる</t>
+          <t>外部副作用の有無と再試行の安全性を説明できる</t>
         </is>
       </c>
       <c r="D5" s="2" t="n"/>
@@ -567,7 +567,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>継続判断</t>
+          <t>継続条件</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -586,12 +586,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>継続判断</t>
+          <t>継続条件</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>ログ / メトリクス / ダンプなど、後追い調査の手がかりがある</t>
+          <t>ログ / メトリクス / ダンプなど、後追い調査の材料が残る</t>
         </is>
       </c>
       <c r="D7" s="2" t="n"/>
@@ -605,12 +605,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>終了判断</t>
+          <t>終了条件</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>途中で何が変わったか分からない場合に、そのまま継続しない</t>
+          <t>途中で何が変わったか不明なときは、継続しない</t>
         </is>
       </c>
       <c r="D8" s="2" t="n"/>
@@ -624,12 +624,12 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>終了判断</t>
+          <t>終了条件</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>共有の書き換え可能な状態の整合が怪しいなら、終了寄りに倒す</t>
+          <t>共有の可変状態の整合が怪しいなら、終了寄りで判断する</t>
         </is>
       </c>
       <c r="D9" s="2" t="n"/>
@@ -643,12 +643,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>終了判断</t>
+          <t>終了条件</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>ロック / キュー / スレッド / 監視ループの寿命管理が壊れている疑いがあるなら、終了寄りに倒す</t>
+          <t>ロック / キュー / スレッド / 監視ループの寿命管理が壊れている疑いがあるなら、終了寄りで判断する</t>
         </is>
       </c>
       <c r="D10" s="2" t="n"/>
@@ -662,12 +662,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>終了判断</t>
+          <t>終了条件</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>外部副作用の重複 / 欠落 / 半端を説明できないなら、終了寄りに倒す</t>
+          <t>外部副作用の重複 / 欠落 / 中途半端な実行を説明できないなら、終了寄りで判断する</t>
         </is>
       </c>
       <c r="D11" s="2" t="n"/>
@@ -681,7 +681,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>終了判断</t>
+          <t>終了条件</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -700,12 +700,12 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>終了判断</t>
+          <t>終了条件</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>ネイティブ境界の破壊やメモリ破壊の疑いを、継続前提で扱わない</t>
+          <t>ネイティブ境界の破損やメモリ破壊の疑いを、継続前提で扱わない</t>
         </is>
       </c>
       <c r="D13" s="2" t="n"/>
@@ -724,7 +724,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>catch (Exception) してログだけ出し、そのまま続けない</t>
+          <t>catch (Exception) してログだけ残し、そのまま続行しない</t>
         </is>
       </c>
       <c r="D14" s="2" t="n"/>
@@ -762,7 +762,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>外部副作用を伴う処理を、再実行安全性なしで盲目的に retry しない</t>
+          <t>外部副作用を伴う処理を、再実行安全性なしで無造作に再試行しない</t>
         </is>
       </c>
       <c r="D16" s="2" t="n"/>
@@ -781,7 +781,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>実際には監視やワーカーループが死んでいるのに、UI だけ生かさない</t>
+          <t>監視やワーカーループが死んだ後に、UI だけを生かさない</t>
         </is>
       </c>
       <c r="D17" s="2" t="n"/>
@@ -800,7 +800,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>クラッシュ回避が重要なら、自動再起動 / セッション復元 / 途中成果保存 / 再実行安全性 / 障害領域分離を先に設計する</t>
+          <t>クラッシュ回避が重要なら、自動再起動 / セッション復元 / 進捗保存 / 再実行安全性 / 障害領域分離を先に設計する</t>
         </is>
       </c>
       <c r="D18" s="2" t="n"/>
@@ -819,7 +819,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>catch する場所を、UI 操作 / 1 リクエスト / 1 ジョブ / 1 接続 / プロセス境界などに寄せる</t>
+          <t>catch する場所を UI 操作 / リクエスト / ジョブ / 接続 / プロセス境界などの境界に寄せる</t>
         </is>
       </c>
       <c r="D19" s="2" t="n"/>
@@ -828,7 +828,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>共有の書き換え可能な状態を、実際的な範囲で小さく保つ</t>
+          <t>想定内の失敗と想定外の例外を別カテゴリで扱う</t>
         </is>
       </c>
       <c r="D20" s="2" t="n"/>
@@ -847,7 +847,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>20</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -857,7 +857,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>被害範囲を小さくしたい危険処理は、別プロセスへ隔離する</t>
+          <t>共有の可変状態は、実務上可能な範囲で小さく保つ</t>
         </is>
       </c>
       <c r="D21" s="2" t="n"/>
@@ -866,7 +866,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -876,7 +876,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>未処理例外フックは、擬似回復より記録と診断を優先する</t>
+          <t>被害範囲を小さくしたい危険処理は、別プロセスへ隔離する</t>
         </is>
       </c>
       <c r="D22" s="2" t="n"/>
@@ -885,7 +885,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -895,7 +895,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>WPF / WinForms の未処理例外イベントで Handled = true にできることを、安全に継続できる証拠としない</t>
+          <t>未処理例外フックでは、擬似回復より記録と診断を優先する</t>
         </is>
       </c>
       <c r="D23" s="2" t="n"/>
@@ -904,17 +904,17 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>23</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>判断順</t>
+          <t>実装方針</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>最初に、失敗した単位を破棄できるかを確認する</t>
+          <t>WPF / WinForms の未処理例外イベントで継続できても、安全とはみなさない</t>
         </is>
       </c>
       <c r="D24" s="2" t="n"/>
@@ -923,7 +923,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>24</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -933,7 +933,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>次に、共有状態を修復または再構築できるかを確認する</t>
+          <t>まず、失敗した単位を破棄できるかを確認する</t>
         </is>
       </c>
       <c r="D25" s="2" t="n"/>
@@ -942,7 +942,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>25</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -952,7 +952,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>次に、外部副作用をまだ説明できるかを確認する</t>
+          <t>次に、共有状態を修復または再構築できるかを確認する</t>
         </is>
       </c>
       <c r="D26" s="2" t="n"/>
@@ -961,7 +961,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>最後に、メモリ / スレッド / ネイティブ境界をまだ信用できるかを確認する</t>
+          <t>次に、外部副作用を説明できるかを確認する</t>
         </is>
       </c>
       <c r="D27" s="2" t="n"/>
@@ -985,17 +985,18 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>???</t>
+          <t>判断順</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>??? / ???? / ?????????????????????</t>
+          <t>最後に、メモリ / スレッド / ネイティブ境界をまだ信用できるかを確認する</t>
         </is>
       </c>
       <c r="D28" s="2" t="n"/>
       <c r="E28" s="2" t="n"/>
     </row>
+    <row r="29"/>
   </sheetData>
   <autoFilter ref="A1:E28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>